<commit_message>
Update support data and sync portal state
</commit_message>
<xml_diff>
--- a/backend/data/current/support_data.xlsx
+++ b/backend/data/current/support_data.xlsx
@@ -35670,12 +35670,12 @@
       </c>
       <c r="J375" t="inlineStr">
         <is>
-          <t>2026-09-17 11:02:11</t>
+          <t>2026-09-17 14:54:17</t>
         </is>
       </c>
       <c r="K375" t="inlineStr">
         <is>
-          <t>2026-09-17 11:02:09</t>
+          <t>2026-09-17 14:54:13</t>
         </is>
       </c>
       <c r="L375" t="inlineStr">
@@ -35688,12 +35688,12 @@
       </c>
       <c r="N375" t="inlineStr">
         <is>
-          <t>{"Open": 1.66, "In Progress": 1.02}</t>
+          <t>{"Open": 1.66, "In Progress": 1.18}</t>
         </is>
       </c>
       <c r="O375" t="inlineStr">
         <is>
-          <t>[{"activity_id": "ACT-CREATE", "actor": "Hassen Chakroun", "action_text": "Ticket created via Email", "timestamp": "2026-09-14T13:09:10Z", "category": "System"}, {"activity_id": "ACT-CONV-0", "actor": "AI Triage Agent", "action_text": "Automated AI triage analysis logged: ? AI Triage ?\ufe0f Label Printing \u00b7 Label/Print Support \u00b7 \u2705 high confidence Summary The KLT label is printing the wrong part number for referenc...", "timestamp": "2026-09-14T13:20:26Z", "category": "Automation"}, {"activity_id": "ACT-FIRSTRESPONSE", "actor": "Agent", "action_text": "First agent response sent", "timestamp": "2026-09-14T13:30:02Z", "category": "Agent"}, {"activity_id": "ACT-CONV-1", "actor": "Agent", "action_text": "Agent reply sent: Hi Hassen Chakroun, Setup is made like that in the system. Kindly help to check with the CS team responsible for thie setup. Ticket: https:/...", "timestamp": "2026-09-14T13:30:02Z", "category": "Reply"}, {"activity_id": "ACT-STATUS", "actor": "System", "action_text": "Status updated to 'In Progress'", "timestamp": "2026-09-16T04:59:13Z", "category": "System"}]</t>
+          <t>[{"activity_id": "ACT-CREATE", "actor": "Hassen Chakroun", "action_text": "Ticket created via Email", "timestamp": "2026-09-14T13:09:10Z", "category": "System"}, {"activity_id": "ACT-CONV-0", "actor": "AI Triage Agent", "action_text": "Automated AI triage analysis logged: ? AI Triage ?\ufe0f Label Printing \u00b7 Label/Print Support \u00b7 \u2705 high confidence Summary The KLT label is printing the wrong part number for referenc...", "timestamp": "2026-09-14T13:20:26Z", "category": "Automation"}, {"activity_id": "ACT-FIRSTRESPONSE", "actor": "Agent", "action_text": "First agent response sent", "timestamp": "2026-09-14T13:30:02Z", "category": "Agent"}, {"activity_id": "ACT-CONV-1", "actor": "Agent", "action_text": "Agent reply sent: Hi Hassen Chakroun, Setup is made like that in the system. Kindly help to check with the CS team responsible for thie setup. Ticket: https:/...", "timestamp": "2026-09-14T13:30:02Z", "category": "Reply"}, {"activity_id": "ACT-STATUS", "actor": "System", "action_text": "Status updated to 'In Progress'", "timestamp": "2026-09-16T04:59:13Z", "category": "System"}, {"activity_id": "ACT-CONV-2", "actor": "Internal Note", "action_text": "Private internal note added: Attaching CR and RFC documents....", "timestamp": "2026-09-17T06:56:26Z", "category": "Note"}, {"activity_id": "ACT-CONV-3", "actor": "Internal Note", "action_text": "Private internal note added: Hi Eric, We have identified a bug in the Germany customer label print program. When there are multiple sales order lines in the shipper, cus...", "timestamp": "2026-09-17T07:26:42Z", "category": "Note"}]</t>
         </is>
       </c>
     </row>
@@ -38500,7 +38500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I121"/>
+  <dimension ref="A1:I123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44185,6 +44185,100 @@
         </is>
       </c>
       <c r="I121" t="inlineStr">
+        <is>
+          <t>Agent logged in successfully</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>AUD-20260917123106929</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>USR-103</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>LOGIN_SUCCESS</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>USR-103</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>2026-09-17 12:31:06</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Agent logged in successfully</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>AUD-20260917145316774</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>USR-101</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>mayur</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>LOGIN_SUCCESS</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>USR-101</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>2026-09-17 14:53:16</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
         <is>
           <t>Agent logged in successfully</t>
         </is>

</xml_diff>